<commit_message>
Refactor of the ReferenceEvent object and connected
</commit_message>
<xml_diff>
--- a/src/cassy/additional_data/templates/path_config_template.xlsx
+++ b/src/cassy/additional_data/templates/path_config_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\laghida\Documents\Github\cassy\src\cassy\additional_data\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3491EAC-79A1-4953-90B4-8FB184B3B827}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBFA7F1F-F48B-485C-B055-226AA750931A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-240" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="-240" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Reference Event Fatigue" sheetId="1" r:id="rId1"/>
@@ -126,9 +126,6 @@
     <t>Is Pressure</t>
   </si>
   <si>
-    <t>Is Occasional</t>
-  </si>
-  <si>
     <t>MPa</t>
   </si>
   <si>
@@ -208,6 +205,9 @@
   </si>
   <si>
     <t>SS316L(N)-IG_SDC-IC</t>
+  </si>
+  <si>
+    <t>Is Short Overstress</t>
   </si>
 </sst>
 </file>
@@ -630,34 +630,34 @@
         <v>7</v>
       </c>
       <c r="B1" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="D1" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="E1" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="F1" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="G1" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="H1" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="I1" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="J1" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="I1" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="J1" s="6" t="s">
+      <c r="K1" s="6" t="s">
         <v>48</v>
-      </c>
-      <c r="K1" s="6" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -665,25 +665,25 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C2" s="10" t="s">
         <v>17</v>
       </c>
       <c r="D2" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="E2" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="E2" s="11" t="s">
+      <c r="F2" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="G2" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="F2" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="G2" s="10" t="s">
+      <c r="H2" s="10" t="s">
         <v>53</v>
-      </c>
-      <c r="H2" s="10" t="s">
-        <v>54</v>
       </c>
       <c r="I2" s="9">
         <v>30000</v>
@@ -700,25 +700,25 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C3" s="10" t="s">
         <v>17</v>
       </c>
       <c r="D3" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="E3" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="E3" s="11" t="s">
+      <c r="F3" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="G3" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="F3" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="G3" s="10" t="s">
+      <c r="H3" s="10" t="s">
         <v>53</v>
-      </c>
-      <c r="H3" s="10" t="s">
-        <v>54</v>
       </c>
       <c r="I3" s="9">
         <v>30000</v>
@@ -870,31 +870,31 @@
         <v>7</v>
       </c>
       <c r="B1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1" t="s">
         <v>41</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>42</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>43</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>44</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>45</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>46</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>48</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -902,25 +902,25 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C2" t="s">
         <v>19</v>
       </c>
       <c r="D2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E2" t="s">
         <v>51</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
+        <v>51</v>
+      </c>
+      <c r="G2" t="s">
         <v>52</v>
       </c>
-      <c r="F2" t="s">
-        <v>52</v>
-      </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>53</v>
-      </c>
-      <c r="H2" t="s">
-        <v>54</v>
       </c>
       <c r="I2" s="3">
         <v>35</v>
@@ -934,25 +934,25 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C3" t="s">
         <v>55</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E3" t="s">
         <v>56</v>
       </c>
-      <c r="D3" t="s">
+      <c r="F3" t="s">
         <v>51</v>
       </c>
-      <c r="E3" t="s">
+      <c r="G3" t="s">
         <v>57</v>
       </c>
-      <c r="F3" t="s">
-        <v>52</v>
-      </c>
-      <c r="G3" t="s">
-        <v>58</v>
-      </c>
       <c r="H3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I3" s="3">
         <v>35</v>
@@ -966,25 +966,25 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C4" t="s">
         <v>19</v>
       </c>
       <c r="D4" t="s">
+        <v>50</v>
+      </c>
+      <c r="E4" t="s">
         <v>51</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G4" t="s">
         <v>52</v>
       </c>
-      <c r="F4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>53</v>
-      </c>
-      <c r="H4" t="s">
-        <v>54</v>
       </c>
       <c r="I4" s="3">
         <v>35</v>
@@ -998,25 +998,25 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C5" t="s">
         <v>55</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
+        <v>50</v>
+      </c>
+      <c r="E5" t="s">
         <v>56</v>
       </c>
-      <c r="D5" t="s">
+      <c r="F5" t="s">
         <v>51</v>
       </c>
-      <c r="E5" t="s">
+      <c r="G5" t="s">
         <v>57</v>
       </c>
-      <c r="F5" t="s">
-        <v>52</v>
-      </c>
-      <c r="G5" t="s">
-        <v>58</v>
-      </c>
       <c r="H5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I5" s="3">
         <v>35</v>
@@ -1079,7 +1079,7 @@
         <v>32</v>
       </c>
       <c r="J1" t="s">
-        <v>33</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -1087,28 +1087,28 @@
         <v>17</v>
       </c>
       <c r="B2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" t="s">
         <v>34</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>35</v>
-      </c>
-      <c r="D2" t="s">
-        <v>36</v>
       </c>
       <c r="E2" s="3">
         <v>1</v>
       </c>
       <c r="G2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H2" t="s">
         <v>37</v>
       </c>
-      <c r="H2" t="s">
-        <v>38</v>
-      </c>
       <c r="I2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="J2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -1116,28 +1116,28 @@
         <v>19</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E3" s="3">
         <v>1</v>
       </c>
       <c r="G3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I3" t="s">
+        <v>36</v>
+      </c>
+      <c r="J3" t="s">
         <v>37</v>
-      </c>
-      <c r="J3" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -1145,10 +1145,10 @@
         <v>21</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D4" t="s">
         <v>22</v>
@@ -1157,19 +1157,19 @@
         <v>0.33</v>
       </c>
       <c r="F4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G4" t="s">
+        <v>36</v>
+      </c>
+      <c r="H4" t="s">
         <v>37</v>
       </c>
-      <c r="H4" t="s">
-        <v>38</v>
-      </c>
       <c r="I4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="J4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -1177,10 +1177,10 @@
         <v>23</v>
       </c>
       <c r="B5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D5" t="s">
         <v>22</v>
@@ -1189,19 +1189,19 @@
         <v>0.33</v>
       </c>
       <c r="F5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H5" t="s">
         <v>37</v>
       </c>
-      <c r="H5" t="s">
-        <v>38</v>
-      </c>
       <c r="I5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="J5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -1209,10 +1209,10 @@
         <v>24</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D6" t="s">
         <v>22</v>
@@ -1221,19 +1221,19 @@
         <v>0.33</v>
       </c>
       <c r="F6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G6" t="s">
+        <v>36</v>
+      </c>
+      <c r="H6" t="s">
         <v>37</v>
       </c>
-      <c r="H6" t="s">
-        <v>38</v>
-      </c>
       <c r="I6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="J6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -1364,7 +1364,7 @@
         <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D2" s="3">
         <v>1</v>
@@ -1381,7 +1381,7 @@
         <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D3" s="3">
         <v>1</v>

</xml_diff>